<commit_message>
Added new RDF data schemes and visual schemes for economy-table124-125, fixed XLSX spreadsheet for economy-table125
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table125.xlsx
+++ b/sources/table_normalization/xlsx/economy-table125.xlsx
@@ -149,7 +149,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -171,6 +171,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -198,7 +204,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -258,11 +264,27 @@
       <alignment horizontal="right" indent="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -792,7 +814,7 @@
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="18" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -958,7 +980,7 @@
       </c>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="19" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="10" t="s">
@@ -1032,26 +1054,26 @@
       </c>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="18"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
+      <c r="A14" s="23"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="17">
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="21">
         <v>13.45</v>
       </c>
-      <c r="G15" s="17">
+      <c r="G15" s="21">
         <v>1037.5999999999999</v>
       </c>
     </row>

</xml_diff>